<commit_message>
Sửa lỗi báo cáo
</commit_message>
<xml_diff>
--- a/src/main/resources/public/BCKCHT_163.xlsx
+++ b/src/main/resources/public/BCKCHT_163.xlsx
@@ -124,7 +124,7 @@
     <t>NĂNG LỰC THÔNG QUA BẾN CẢNG, CẦU CẢNG</t>
   </si>
   <si>
-    <t>Danh mục bến cảng, cầu cảng</t>
+    <t>Danh mục bến cảng, cầu cảng, cảng bến thủy nội địa</t>
   </si>
   <si>
     <t>A</t>
@@ -154,10 +154,10 @@
     <t>Chiều dài bến cảng, cầu cảng (m)</t>
   </si>
   <si>
-    <t>Tổng diện tích (ha)</t>
-  </si>
-  <si>
     <t>Tàu neo đậu, làm hàng lớn nhất (DWT)</t>
+  </si>
+  <si>
+    <t>Ghi chú</t>
   </si>
   <si>
     <t>(Ký, ghi rõ họ tên)</t>
@@ -754,7 +754,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" mc:Ignorable="x14ac">
+<worksheet xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" mc:Ignorable="x14ac">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>

</xml_diff>